<commit_message>
fix(linzess): improve sitemap SEO (proper description + canonical)
The sitemap's auto meta description was the ISI legal copy (the first
long paragraph), and the page had no canonical. Add a curated per-page
sitemap description and a canonical URL in the utility metadata
transformer, then re-import the sitemap.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-linzess-utility.report.xlsx
+++ b/tools/importer/reports/import-linzess-utility.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="46">
   <si>
     <t>_reportFile</t>
   </si>
@@ -82,7 +82,7 @@
     <t>savings-card/terms</t>
   </si>
   <si>
-    <t>2026-06-05T06:49:16.045Z</t>
+    <t>2026-06-19T10:37:46.341Z</t>
   </si>
   <si>
     <t/>
@@ -91,6 +91,15 @@
     <t>https://www.linzess.com/savings-card/terms</t>
   </si>
   <si>
+    <t>linzess/savings-card/terms.report.json</t>
+  </si>
+  <si>
+    <t>linzess/savings-card/terms</t>
+  </si>
+  <si>
+    <t>2026-06-19T10:41:01.005Z</t>
+  </si>
+  <si>
     <t>linzess/utility/es-home.report.json</t>
   </si>
   <si>
@@ -133,7 +142,7 @@
     <t>linzess/utility/sitemap</t>
   </si>
   <si>
-    <t>2026-06-19T08:36:13.870Z</t>
+    <t>2026-06-19T10:53:24.531Z</t>
   </si>
   <si>
     <t>Sitemap | LINZESS® (linaclotide)</t>
@@ -528,7 +537,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
@@ -648,77 +657,103 @@
         <v>26</v>
       </c>
       <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
         <v>27</v>
-      </c>
-      <c r="C5" t="s">
-        <v>28</v>
       </c>
       <c r="D5" t="s">
         <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="F5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G5" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="H5" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
       </c>
       <c r="E6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" t="s">
         <v>35</v>
-      </c>
-      <c r="F6" t="s">
-        <v>36</v>
-      </c>
-      <c r="G6" t="s">
-        <v>24</v>
-      </c>
-      <c r="H6" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B7" t="s">
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
       </c>
       <c r="E7" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" t="s">
         <v>40</v>
       </c>
-      <c r="G7" t="s">
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>41</v>
       </c>
-      <c r="H7" t="s">
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
         <v>42</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" t="s">
+        <v>44</v>
+      </c>
+      <c r="H8" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>